<commit_message>
Prix et familles de pièces donnés par Emmanuelle
- Cinq familles : naissance (doudou et cadre), linge de maison, dentelle
  libre, fêtes et évènements, sacs et trousses cousus main
- Prix « à partir de » : 8, 8, 12, 10 et 20 € ; délai 8 à 15 jours partout
- Le délai accepte un intervalle (« 8 à 15 ») : contenu, admin, import
- Budgets du formulaire ajustés (moins de 20 €…)
- Questionnaire régénéré avec ces valeurs

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017vDojrqUxLfCDyDEvVKxZw
</commit_message>
<xml_diff>
--- a/docs/questionnaire-emma-broderie.xlsx
+++ b/docs/questionnaire-emma-broderie.xlsx
@@ -1290,19 +1290,21 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>L'arbre de vie en dentelle</t>
+          <t>Pièces en dentelle libre</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>L'arbre de vie en dentelle</t>
+          <t>Pièces en dentelle libre</t>
         </is>
       </c>
       <c r="D4" s="9" t="n">
-        <v>38</v>
-      </c>
-      <c r="E4" s="9" t="n">
-        <v>14</v>
+        <v>12</v>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>8 à 15</t>
+        </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
@@ -1331,10 +1333,12 @@
         </is>
       </c>
       <c r="D5" s="9" t="n">
-        <v>45</v>
-      </c>
-      <c r="E5" s="9" t="n">
-        <v>12</v>
+        <v>8</v>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>8 à 15</t>
+        </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
@@ -1354,19 +1358,21 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>La chaussette de Noël</t>
+          <t>Fêtes et évènements</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>La chaussette de Noël</t>
+          <t>Fêtes et évènements</t>
         </is>
       </c>
       <c r="D6" s="9" t="n">
-        <v>26</v>
-      </c>
-      <c r="E6" s="9" t="n">
         <v>10</v>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>8 à 15</t>
+        </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -1386,19 +1392,21 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Le doudou de naissance</t>
+          <t>Doudou et cadre de naissance</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Le doudou de naissance</t>
+          <t>Doudou et cadre de naissance</t>
         </is>
       </c>
       <c r="D7" s="9" t="n">
-        <v>32</v>
-      </c>
-      <c r="E7" s="9" t="n">
-        <v>10</v>
+        <v>8</v>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>8 à 15</t>
+        </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
@@ -1418,19 +1426,21 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Le drap de bain au prénom</t>
+          <t>Serviettes et linge au prénom</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Le drap de bain au prénom</t>
+          <t>Serviettes et linge au prénom</t>
         </is>
       </c>
       <c r="D8" s="9" t="n">
-        <v>24</v>
-      </c>
-      <c r="E8" s="9" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>8 à 15</t>
+        </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
@@ -1450,19 +1460,21 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>La trousse cousue main</t>
+          <t>Sacs et trousses cousus main</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>La trousse cousue main</t>
+          <t>Sacs et trousses cousus main</t>
         </is>
       </c>
       <c r="D9" s="9" t="n">
-        <v>28</v>
-      </c>
-      <c r="E9" s="9" t="n">
-        <v>10</v>
+        <v>20</v>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>8 à 15</t>
+        </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Premier retour du questionnaire d'Emmanuelle
- Coordonnées réelles : téléphone et WhatsApp, e-mail, nom légal, SIRET
- Cinq familles dans son ordre, avec ses titres et descriptions ; la carte
  affiche la description à la place de l'étiquette de catégorie
- Noël : commandes jusqu'au 10 décembre (calendrier, FAQ, fiches)
- Paiement : virement, espèces ou Wero
- Couture : ajout des petites retouches (ourlets de pantalon)
- Mentions légales : SIRET, nom et commune renseignés ; restent l'adresse
  du siège et le régime de TVA
- Questionnaire : onglet créations plus clair (une ligne = une carte)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017vDojrqUxLfCDyDEvVKxZw
</commit_message>
<xml_diff>
--- a/docs/questionnaire-emma-broderie.xlsx
+++ b/docs/questionnaire-emma-broderie.xlsx
@@ -1213,7 +1213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1236,7 +1236,7 @@
     <row r="2">
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>Corrigez le nom, le prix et le délai. Les valeurs déjà inscrites sont des exemples à vérifier.</t>
+          <t>Une ligne = une carte du site. Ne touchez pas à la colonne « Carte actuelle » : modifiez seulement les cases jaunes de la même ligne.</t>
         </is>
       </c>
     </row>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Création</t>
+          <t>Carte actuelle (ne pas modifier)</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -1285,21 +1285,21 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>arbre-de-vie-dentelle</t>
+          <t>drap-de-bain-brode-prenom</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Pièces en dentelle libre</t>
+          <t>Linge de maison</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Pièces en dentelle libre</t>
+          <t>Linge de maison</t>
         </is>
       </c>
       <c r="D4" s="9" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
@@ -1319,17 +1319,17 @@
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>cadre-naissance-brode</t>
+          <t>doudou-lapin-brode-prenom</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Le cadre de naissance</t>
+          <t>Naissance et doudou</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Le cadre de naissance</t>
+          <t>Naissance et doudou</t>
         </is>
       </c>
       <c r="D5" s="9" t="n">
@@ -1353,21 +1353,21 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>chaussette-noel-brodee</t>
+          <t>arbre-de-vie-dentelle</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Fêtes et évènements</t>
+          <t>Dentelle libre</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Fêtes et évènements</t>
+          <t>Dentelle libre</t>
         </is>
       </c>
       <c r="D6" s="9" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
@@ -1380,28 +1380,28 @@
         </is>
       </c>
       <c r="G6" s="9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H6" s="9" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>doudou-lapin-brode-prenom</t>
+          <t>chaussette-noel-brodee</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Doudou et cadre de naissance</t>
+          <t>Fêtes et évènements</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Doudou et cadre de naissance</t>
+          <t>Fêtes et évènements</t>
         </is>
       </c>
       <c r="D7" s="9" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
@@ -1414,28 +1414,28 @@
         </is>
       </c>
       <c r="G7" s="9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H7" s="9" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>drap-de-bain-brode-prenom</t>
+          <t>trousse-cousue-brodee</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Serviettes et linge au prénom</t>
+          <t>Couture</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Serviettes et linge au prénom</t>
+          <t>Couture</t>
         </is>
       </c>
       <c r="D8" s="9" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
@@ -1448,47 +1448,13 @@
         </is>
       </c>
       <c r="G8" s="9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H8" s="9" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>trousse-cousue-brodee</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Sacs et trousses cousus main</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>Sacs et trousses cousus main</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>8 à 15</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Oui</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="H9" s="9" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F4:F9" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisissez dans la liste." prompt="Choisissez dans la liste" type="list">
+    <dataValidation sqref="F4:F8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Choisissez dans la liste." prompt="Choisissez dans la liste" type="list">
       <formula1>"Oui,Non"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>